<commit_message>
Deduplicate + modificari workflow de test
</commit_message>
<xml_diff>
--- a/Job_Scraping_Project/Data/Output/Jobs.xlsx
+++ b/Job_Scraping_Project/Data/Output/Jobs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ana\Documents\facultate\ANUL III\rpa\Job_Scraping_RPAUiPath_Project\Job_Scraping_Project\Data\Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B23DB07-BFA3-408C-A202-0D9B0C133B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD7CB697-4524-46D2-8F26-13AEB8281250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" firstSheet="0" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
@@ -26,34 +26,145 @@
     <x:t>Keyword</x:t>
   </x:si>
   <x:si>
-    <x:t>Location</x:t>
+    <x:t>Site</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JobTitle</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Company</x:t>
+  </x:si>
+  <x:si>
+    <x:t>City</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Salary</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JobUrl</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ScrapeDate</x:t>
   </x:si>
   <x:si>
     <x:t>QA Engineer</x:t>
   </x:si>
   <x:si>
+    <x:t>eJobs</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TechSoft SRL</x:t>
+  </x:si>
+  <x:si>
     <x:t>Remote</x:t>
   </x:si>
   <x:si>
+    <x:t>6000-8000 RON</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://example.com/jobs/qa-engineer-techsoft-001</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-01-02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BestJobs</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Manual QA Tester</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CloudNova</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Bucuresti</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>https://example.com/jobs/manual-qa-cloudnova-014</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-01-01</x:t>
+  </x:si>
+  <x:si>
     <x:t>RPA Developer</x:t>
   </x:si>
   <x:si>
-    <x:t>Bucharest</x:t>
+    <x:t>RPA Developer (UiPath)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AutomationHub</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cluj-Napoca</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9000-12000 RON</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://example.com/jobs/rpa-developer-automationhub-210</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Negotiable</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://example.com/jobs/rpa-developer-automationhub-211</x:t>
   </x:si>
   <x:si>
     <x:t>.NET Developer</x:t>
   </x:si>
   <x:si>
-    <x:t>Java Developer</x:t>
-  </x:si>
-  <x:si>
-    <x:t>C++ Developer</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Python Developer</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cloud Engineer</x:t>
+    <x:t>FinApps</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12000-16000 RON</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://example.com/jobs/dotnet-finapps-077</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2025-12-31</x:t>
+  </x:si>
+  <x:si>
+    <x:t>.NET Developer (C#)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://example.com/jobs/dotnet-finapps-078</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QA Automation Engineer</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PixelWorks</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Timisoara</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7000-10000 RON</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://example.com/jobs/qa-auto-pixelworks-032</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Data Analyst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Junior Data Analyst</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DataSpring</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Iasi</x:t>
+  </x:si>
+  <x:si>
+    <x:t>5000-6500 RON</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://example.com/jobs/jr-data-analyst-dataspring-055</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -397,74 +508,247 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:B7"/>
+  <x:dimension ref="A1:H9"/>
   <x:sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <x:cols>
-    <x:col min="1" max="1" width="13.664062" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="21.886719" style="0" customWidth="1"/>
+    <x:col min="2" max="6" width="9.109375" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="74.886719" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="19.109375" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <x:row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <x:c r="A1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
         <x:v>1</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <x:c r="C1" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D1" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E1" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F1" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G1" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H1" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <x:c r="A2" s="0" t="s">
-        <x:v>2</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:2" x14ac:dyDescent="0.3">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <x:c r="A3" s="0" t="s">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <x:c r="A4" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <x:c r="A5" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H5" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <x:c r="A6" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="H6" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <x:c r="A7" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="H7" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <x:c r="A8" s="0" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <x:c r="A7" s="0" t="s">
+      <x:c r="B8" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:2">
-      <x:c r="A8" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>5</x:v>
+      <x:c r="C8" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="H8" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <x:c r="A9" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="H9" s="0" t="s">
+        <x:v>14</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>